<commit_message>
chore(auto): claude session checkpoint (17 file(s), 2026-04-27T00:12:02Z)
</commit_message>
<xml_diff>
--- a/tests/regression_artifacts/downloads/email_TSCW18489131_budget_marine_grenada/current/0098813384.xlsx
+++ b/tests/regression_artifacts/downloads/email_TSCW18489131_budget_marine_grenada/current/0098813384.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invoice Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Invoice Data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM87"/>
+  <dimension ref="A1:AM88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1093,12 +1093,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Footwear</t>
+          <t>Yachts &amp; Other Vessels</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>89069000</t>
+          <t>89039900</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -1157,7 +1157,7 @@
       <c r="AJ6" s="2" t="n"/>
       <c r="AK6" s="2" t="inlineStr">
         <is>
-          <t>89069000</t>
+          <t>89039900</t>
         </is>
       </c>
     </row>
@@ -1176,12 +1176,12 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Footwear</t>
+          <t>Yachts &amp; Other Vessels</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>89069000</t>
+          <t>89039900</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
@@ -1240,7 +1240,7 @@
       <c r="AJ7" s="2" t="n"/>
       <c r="AK7" s="2" t="inlineStr">
         <is>
-          <t>89069000</t>
+          <t>89039900</t>
         </is>
       </c>
     </row>
@@ -1259,12 +1259,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Footwear</t>
+          <t>Yachts &amp; Other Vessels</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>89069000</t>
+          <t>89039900</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
@@ -1323,7 +1323,7 @@
       <c r="AJ8" s="2" t="n"/>
       <c r="AK8" s="2" t="inlineStr">
         <is>
-          <t>89069000</t>
+          <t>89039900</t>
         </is>
       </c>
     </row>
@@ -1342,12 +1342,12 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Footwear</t>
+          <t>Yachts &amp; Other Vessels</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>89069000</t>
+          <t>89039900</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
@@ -1406,7 +1406,7 @@
       <c r="AJ9" s="2" t="n"/>
       <c r="AK9" s="2" t="inlineStr">
         <is>
-          <t>89069000</t>
+          <t>89039900</t>
         </is>
       </c>
     </row>
@@ -1425,12 +1425,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Footwear</t>
+          <t>Yachts &amp; Other Vessels</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>89069000</t>
+          <t>89039900</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -1489,7 +1489,7 @@
       <c r="AJ10" s="2" t="n"/>
       <c r="AK10" s="2" t="inlineStr">
         <is>
-          <t>89069000</t>
+          <t>89039900</t>
         </is>
       </c>
     </row>
@@ -1508,12 +1508,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Footwear</t>
+          <t>Yachts &amp; Other Vessels</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>89069000</t>
+          <t>89039900</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
@@ -1572,7 +1572,7 @@
       <c r="AJ11" s="2" t="n"/>
       <c r="AK11" s="2" t="inlineStr">
         <is>
-          <t>89069000</t>
+          <t>89039900</t>
         </is>
       </c>
     </row>
@@ -1591,12 +1591,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Footwear</t>
+          <t>Yachts &amp; Other Vessels</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>89069000</t>
+          <t>89039900</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
@@ -1655,7 +1655,7 @@
       <c r="AJ12" s="2" t="n"/>
       <c r="AK12" s="2" t="inlineStr">
         <is>
-          <t>89069000</t>
+          <t>89039900</t>
         </is>
       </c>
     </row>
@@ -1674,12 +1674,12 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Footwear</t>
+          <t>Yachts &amp; Other Vessels</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>89069000</t>
+          <t>89039900</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
@@ -1738,7 +1738,7 @@
       <c r="AJ13" s="2" t="n"/>
       <c r="AK13" s="2" t="inlineStr">
         <is>
-          <t>89069000</t>
+          <t>89039900</t>
         </is>
       </c>
     </row>
@@ -3168,12 +3168,12 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Other Covering the ankle but not covering the knee</t>
+          <t>Footwear</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>64019290</t>
+          <t>64039990</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr"/>
@@ -3232,7 +3232,7 @@
       <c r="AJ31" s="2" t="n"/>
       <c r="AK31" s="2" t="inlineStr">
         <is>
-          <t>64019290</t>
+          <t>64039990</t>
         </is>
       </c>
     </row>
@@ -3251,12 +3251,12 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Other Covering the ankle but not covering the knee</t>
+          <t>Footwear</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>64019290</t>
+          <t>64039990</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr"/>
@@ -3315,7 +3315,7 @@
       <c r="AJ32" s="2" t="n"/>
       <c r="AK32" s="2" t="inlineStr">
         <is>
-          <t>64019290</t>
+          <t>64039990</t>
         </is>
       </c>
     </row>
@@ -3334,12 +3334,12 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Other Covering the ankle but not covering the knee</t>
+          <t>Footwear</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>64019290</t>
+          <t>64039990</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr"/>
@@ -3398,7 +3398,7 @@
       <c r="AJ33" s="2" t="n"/>
       <c r="AK33" s="2" t="inlineStr">
         <is>
-          <t>64019290</t>
+          <t>64039990</t>
         </is>
       </c>
     </row>
@@ -3417,12 +3417,12 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Other Covering the ankle but not covering the knee</t>
+          <t>Footwear</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>64019290</t>
+          <t>64039990</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr"/>
@@ -3481,7 +3481,7 @@
       <c r="AJ34" s="2" t="n"/>
       <c r="AK34" s="2" t="inlineStr">
         <is>
-          <t>64019290</t>
+          <t>64039990</t>
         </is>
       </c>
     </row>
@@ -3500,12 +3500,12 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Other Covering the ankle but not covering the knee</t>
+          <t>Footwear</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>64019290</t>
+          <t>64039990</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr"/>
@@ -3564,7 +3564,7 @@
       <c r="AJ35" s="2" t="n"/>
       <c r="AK35" s="2" t="inlineStr">
         <is>
-          <t>64019290</t>
+          <t>64039990</t>
         </is>
       </c>
     </row>
@@ -3583,12 +3583,12 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Other Covering the ankle but not covering the knee</t>
+          <t>Footwear</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>64019290</t>
+          <t>64039990</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr"/>
@@ -3647,7 +3647,7 @@
       <c r="AJ36" s="2" t="n"/>
       <c r="AK36" s="2" t="inlineStr">
         <is>
-          <t>64019290</t>
+          <t>64039990</t>
         </is>
       </c>
     </row>
@@ -3666,12 +3666,12 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Other Covering the ankle but not covering the knee</t>
+          <t>Footwear</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>64019290</t>
+          <t>64039990</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr"/>
@@ -3730,7 +3730,7 @@
       <c r="AJ37" s="2" t="n"/>
       <c r="AK37" s="2" t="inlineStr">
         <is>
-          <t>64019290</t>
+          <t>64039990</t>
         </is>
       </c>
     </row>
@@ -3749,12 +3749,12 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Other Covering the ankle but not covering the knee</t>
+          <t>Footwear</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>64019290</t>
+          <t>64039990</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr"/>
@@ -3813,7 +3813,7 @@
       <c r="AJ38" s="2" t="n"/>
       <c r="AK38" s="2" t="inlineStr">
         <is>
-          <t>64019290</t>
+          <t>64039990</t>
         </is>
       </c>
     </row>
@@ -4247,12 +4247,12 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Singlets and other vests</t>
+          <t>Wine of Fresh Grapes</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>61091020</t>
+          <t>22042990</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr"/>
@@ -4311,7 +4311,7 @@
       <c r="AJ44" s="2" t="n"/>
       <c r="AK44" s="2" t="inlineStr">
         <is>
-          <t>61091020</t>
+          <t>22042990</t>
         </is>
       </c>
     </row>
@@ -4330,12 +4330,12 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Singlets and other vests</t>
+          <t>Wine of Fresh Grapes</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>61091020</t>
+          <t>22042990</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr"/>
@@ -4394,7 +4394,7 @@
       <c r="AJ45" s="2" t="n"/>
       <c r="AK45" s="2" t="inlineStr">
         <is>
-          <t>61091020</t>
+          <t>22042990</t>
         </is>
       </c>
     </row>
@@ -4413,12 +4413,12 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Singlets and other vests</t>
+          <t>Wine of Fresh Grapes</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>61091020</t>
+          <t>22042990</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr"/>
@@ -4477,7 +4477,7 @@
       <c r="AJ46" s="2" t="n"/>
       <c r="AK46" s="2" t="inlineStr">
         <is>
-          <t>61091020</t>
+          <t>22042990</t>
         </is>
       </c>
     </row>
@@ -4496,12 +4496,12 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Singlets and other vests</t>
+          <t>Wine of Fresh Grapes</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>61091020</t>
+          <t>22042990</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr"/>
@@ -4560,7 +4560,7 @@
       <c r="AJ47" s="2" t="n"/>
       <c r="AK47" s="2" t="inlineStr">
         <is>
-          <t>61091020</t>
+          <t>22042990</t>
         </is>
       </c>
     </row>
@@ -4579,12 +4579,12 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Singlets and other vests</t>
+          <t>Wine of Fresh Grapes</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>61091020</t>
+          <t>22042990</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr"/>
@@ -4643,7 +4643,7 @@
       <c r="AJ48" s="2" t="n"/>
       <c r="AK48" s="2" t="inlineStr">
         <is>
-          <t>61091020</t>
+          <t>22042990</t>
         </is>
       </c>
     </row>
@@ -5907,12 +5907,12 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Footwear</t>
+          <t>WATER SPORTS</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>06029090</t>
+          <t>95062900</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr"/>
@@ -5971,7 +5971,7 @@
       <c r="AJ64" s="2" t="n"/>
       <c r="AK64" s="2" t="inlineStr">
         <is>
-          <t>06029090</t>
+          <t>95062900</t>
         </is>
       </c>
     </row>
@@ -5990,12 +5990,12 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>Footwear</t>
+          <t>WATER SPORTS</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>06029090</t>
+          <t>95062900</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr"/>
@@ -6054,7 +6054,7 @@
       <c r="AJ65" s="2" t="n"/>
       <c r="AK65" s="2" t="inlineStr">
         <is>
-          <t>06029090</t>
+          <t>95062900</t>
         </is>
       </c>
     </row>
@@ -6073,12 +6073,12 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Footwear</t>
+          <t>WATER SPORTS</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>06029090</t>
+          <t>95062900</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr"/>
@@ -6137,7 +6137,7 @@
       <c r="AJ66" s="2" t="n"/>
       <c r="AK66" s="2" t="inlineStr">
         <is>
-          <t>06029090</t>
+          <t>95062900</t>
         </is>
       </c>
     </row>
@@ -6156,12 +6156,12 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Footwear</t>
+          <t>WATER SPORTS</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>06029090</t>
+          <t>95062900</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr"/>
@@ -6220,7 +6220,7 @@
       <c r="AJ67" s="2" t="n"/>
       <c r="AK67" s="2" t="inlineStr">
         <is>
-          <t>06029090</t>
+          <t>95062900</t>
         </is>
       </c>
     </row>
@@ -6239,12 +6239,12 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Footwear</t>
+          <t>WATER SPORTS</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>06029090</t>
+          <t>95062900</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr"/>
@@ -6303,7 +6303,7 @@
       <c r="AJ68" s="2" t="n"/>
       <c r="AK68" s="2" t="inlineStr">
         <is>
-          <t>06029090</t>
+          <t>95062900</t>
         </is>
       </c>
     </row>
@@ -6636,7 +6636,7 @@
       <c r="I77" s="7" t="n"/>
       <c r="J77" s="8" t="inlineStr">
         <is>
-          <t>CET (weighted avg 17.1%)</t>
+          <t>CET (weighted avg 20.0%)</t>
         </is>
       </c>
       <c r="K77" s="7" t="n"/>
@@ -6645,7 +6645,7 @@
       <c r="N77" s="7" t="n"/>
       <c r="O77" s="7" t="n"/>
       <c r="P77" s="9" t="n">
-        <v>2065.54</v>
+        <v>2422.8</v>
       </c>
       <c r="Q77" s="7" t="n"/>
       <c r="R77" s="7" t="n"/>
@@ -6681,7 +6681,7 @@
       <c r="I78" s="7" t="n"/>
       <c r="J78" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  └ 06029090: 0% CET (5% of value)</t>
+          <t xml:space="preserve">  └ 22042990: 20% CET (7% of value)</t>
         </is>
       </c>
       <c r="K78" s="7" t="n"/>
@@ -6690,7 +6690,7 @@
       <c r="N78" s="7" t="n"/>
       <c r="O78" s="7" t="n"/>
       <c r="P78" s="9" t="n">
-        <v>0</v>
+        <v>172.47</v>
       </c>
       <c r="Q78" s="7" t="n"/>
       <c r="R78" s="7" t="n"/>
@@ -6726,7 +6726,7 @@
       <c r="I79" s="7" t="n"/>
       <c r="J79" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  └ 61091020: 20% CET (20% of value)</t>
+          <t xml:space="preserve">  └ 61091020: 20% CET (13% of value)</t>
         </is>
       </c>
       <c r="K79" s="7" t="n"/>
@@ -6735,7 +6735,7 @@
       <c r="N79" s="7" t="n"/>
       <c r="O79" s="7" t="n"/>
       <c r="P79" s="9" t="n">
-        <v>492.77</v>
+        <v>320.3</v>
       </c>
       <c r="Q79" s="7" t="n"/>
       <c r="R79" s="7" t="n"/>
@@ -6771,7 +6771,7 @@
       <c r="I80" s="7" t="n"/>
       <c r="J80" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  └ 64019290: 20% CET (9% of value)</t>
+          <t xml:space="preserve">  └ 64029910: 20% CET (46% of value)</t>
         </is>
       </c>
       <c r="K80" s="7" t="n"/>
@@ -6780,7 +6780,7 @@
       <c r="N80" s="7" t="n"/>
       <c r="O80" s="7" t="n"/>
       <c r="P80" s="9" t="n">
-        <v>219.01</v>
+        <v>1123.79</v>
       </c>
       <c r="Q80" s="7" t="n"/>
       <c r="R80" s="7" t="n"/>
@@ -6816,7 +6816,7 @@
       <c r="I81" s="7" t="n"/>
       <c r="J81" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  └ 64029910: 20% CET (46% of value)</t>
+          <t xml:space="preserve">  └ 64039990: 20% CET (9% of value)</t>
         </is>
       </c>
       <c r="K81" s="7" t="n"/>
@@ -6825,7 +6825,7 @@
       <c r="N81" s="7" t="n"/>
       <c r="O81" s="7" t="n"/>
       <c r="P81" s="9" t="n">
-        <v>1123.79</v>
+        <v>219.01</v>
       </c>
       <c r="Q81" s="7" t="n"/>
       <c r="R81" s="7" t="n"/>
@@ -6861,7 +6861,7 @@
       <c r="I82" s="7" t="n"/>
       <c r="J82" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  └ 89069000: 5% CET (14% of value)</t>
+          <t xml:space="preserve">  └ 89039900: 20% CET (14% of value)</t>
         </is>
       </c>
       <c r="K82" s="7" t="n"/>
@@ -6870,7 +6870,7 @@
       <c r="N82" s="7" t="n"/>
       <c r="O82" s="7" t="n"/>
       <c r="P82" s="9" t="n">
-        <v>82.13</v>
+        <v>328.51</v>
       </c>
       <c r="Q82" s="7" t="n"/>
       <c r="R82" s="7" t="n"/>
@@ -6951,7 +6951,7 @@
       <c r="I84" s="7" t="n"/>
       <c r="J84" s="8" t="inlineStr">
         <is>
-          <t>CSC (6%)</t>
+          <t xml:space="preserve">  └ 95062900: 20% CET (5% of value)</t>
         </is>
       </c>
       <c r="K84" s="7" t="n"/>
@@ -6960,7 +6960,7 @@
       <c r="N84" s="7" t="n"/>
       <c r="O84" s="7" t="n"/>
       <c r="P84" s="9" t="n">
-        <v>726.84</v>
+        <v>110.87</v>
       </c>
       <c r="Q84" s="7" t="n"/>
       <c r="R84" s="7" t="n"/>
@@ -6996,7 +6996,7 @@
       <c r="I85" s="7" t="n"/>
       <c r="J85" s="8" t="inlineStr">
         <is>
-          <t>VAT (15%) on CIF+CET+CSC</t>
+          <t>CSC (6%)</t>
         </is>
       </c>
       <c r="K85" s="7" t="n"/>
@@ -7005,7 +7005,7 @@
       <c r="N85" s="7" t="n"/>
       <c r="O85" s="7" t="n"/>
       <c r="P85" s="9" t="n">
-        <v>2235.95</v>
+        <v>726.84</v>
       </c>
       <c r="Q85" s="7" t="n"/>
       <c r="R85" s="7" t="n"/>
@@ -7030,94 +7030,139 @@
       <c r="AK85" s="7" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="10" t="n"/>
-      <c r="B86" s="10" t="n"/>
-      <c r="C86" s="10" t="n"/>
-      <c r="D86" s="10" t="n"/>
-      <c r="E86" s="10" t="n"/>
-      <c r="F86" s="10" t="n"/>
-      <c r="G86" s="10" t="n"/>
-      <c r="H86" s="10" t="n"/>
-      <c r="I86" s="10" t="n"/>
-      <c r="J86" s="6" t="inlineStr">
+      <c r="A86" s="7" t="n"/>
+      <c r="B86" s="7" t="n"/>
+      <c r="C86" s="7" t="n"/>
+      <c r="D86" s="7" t="n"/>
+      <c r="E86" s="7" t="n"/>
+      <c r="F86" s="7" t="n"/>
+      <c r="G86" s="7" t="n"/>
+      <c r="H86" s="7" t="n"/>
+      <c r="I86" s="7" t="n"/>
+      <c r="J86" s="8" t="inlineStr">
+        <is>
+          <t>VAT (15%) on CIF+CET+CSC</t>
+        </is>
+      </c>
+      <c r="K86" s="7" t="n"/>
+      <c r="L86" s="7" t="n"/>
+      <c r="M86" s="7" t="n"/>
+      <c r="N86" s="7" t="n"/>
+      <c r="O86" s="7" t="n"/>
+      <c r="P86" s="9" t="n">
+        <v>2289.54</v>
+      </c>
+      <c r="Q86" s="7" t="n"/>
+      <c r="R86" s="7" t="n"/>
+      <c r="S86" s="7" t="n"/>
+      <c r="T86" s="7" t="n"/>
+      <c r="U86" s="7" t="n"/>
+      <c r="V86" s="7" t="n"/>
+      <c r="W86" s="7" t="n"/>
+      <c r="X86" s="7" t="n"/>
+      <c r="Y86" s="7" t="n"/>
+      <c r="Z86" s="7" t="n"/>
+      <c r="AA86" s="7" t="n"/>
+      <c r="AB86" s="7" t="n"/>
+      <c r="AC86" s="7" t="n"/>
+      <c r="AD86" s="7" t="n"/>
+      <c r="AE86" s="7" t="n"/>
+      <c r="AF86" s="7" t="n"/>
+      <c r="AG86" s="7" t="n"/>
+      <c r="AH86" s="7" t="n"/>
+      <c r="AI86" s="7" t="n"/>
+      <c r="AJ86" s="7" t="n"/>
+      <c r="AK86" s="7" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="10" t="n"/>
+      <c r="B87" s="10" t="n"/>
+      <c r="C87" s="10" t="n"/>
+      <c r="D87" s="10" t="n"/>
+      <c r="E87" s="10" t="n"/>
+      <c r="F87" s="10" t="n"/>
+      <c r="G87" s="10" t="n"/>
+      <c r="H87" s="10" t="n"/>
+      <c r="I87" s="10" t="n"/>
+      <c r="J87" s="6" t="inlineStr">
         <is>
           <t>ESTIMATED TOTAL DUTIES</t>
         </is>
       </c>
-      <c r="K86" s="10" t="n"/>
-      <c r="L86" s="10" t="n"/>
-      <c r="M86" s="10" t="n"/>
-      <c r="N86" s="10" t="n"/>
-      <c r="O86" s="10" t="n"/>
-      <c r="P86" s="11" t="n">
-        <v>5028.33</v>
-      </c>
-      <c r="Q86" s="10" t="n"/>
-      <c r="R86" s="10" t="n"/>
-      <c r="S86" s="10" t="n"/>
-      <c r="T86" s="10" t="n"/>
-      <c r="U86" s="10" t="n"/>
-      <c r="V86" s="10" t="n"/>
-      <c r="W86" s="10" t="n"/>
-      <c r="X86" s="10" t="n"/>
-      <c r="Y86" s="10" t="n"/>
-      <c r="Z86" s="10" t="n"/>
-      <c r="AA86" s="10" t="n"/>
-      <c r="AB86" s="10" t="n"/>
-      <c r="AC86" s="10" t="n"/>
-      <c r="AD86" s="10" t="n"/>
-      <c r="AE86" s="10" t="n"/>
-      <c r="AF86" s="10" t="n"/>
-      <c r="AG86" s="10" t="n"/>
-      <c r="AH86" s="10" t="n"/>
-      <c r="AI86" s="10" t="n"/>
-      <c r="AJ86" s="10" t="n"/>
-      <c r="AK86" s="10" t="n"/>
-    </row>
-    <row r="87">
-      <c r="A87" s="7" t="n"/>
-      <c r="B87" s="7" t="n"/>
-      <c r="C87" s="7" t="n"/>
-      <c r="D87" s="7" t="n"/>
-      <c r="E87" s="7" t="n"/>
-      <c r="F87" s="7" t="n"/>
-      <c r="G87" s="7" t="n"/>
-      <c r="H87" s="7" t="n"/>
-      <c r="I87" s="7" t="n"/>
-      <c r="J87" s="8" t="inlineStr">
+      <c r="K87" s="10" t="n"/>
+      <c r="L87" s="10" t="n"/>
+      <c r="M87" s="10" t="n"/>
+      <c r="N87" s="10" t="n"/>
+      <c r="O87" s="10" t="n"/>
+      <c r="P87" s="11" t="n">
+        <v>5439.18</v>
+      </c>
+      <c r="Q87" s="10" t="n"/>
+      <c r="R87" s="10" t="n"/>
+      <c r="S87" s="10" t="n"/>
+      <c r="T87" s="10" t="n"/>
+      <c r="U87" s="10" t="n"/>
+      <c r="V87" s="10" t="n"/>
+      <c r="W87" s="10" t="n"/>
+      <c r="X87" s="10" t="n"/>
+      <c r="Y87" s="10" t="n"/>
+      <c r="Z87" s="10" t="n"/>
+      <c r="AA87" s="10" t="n"/>
+      <c r="AB87" s="10" t="n"/>
+      <c r="AC87" s="10" t="n"/>
+      <c r="AD87" s="10" t="n"/>
+      <c r="AE87" s="10" t="n"/>
+      <c r="AF87" s="10" t="n"/>
+      <c r="AG87" s="10" t="n"/>
+      <c r="AH87" s="10" t="n"/>
+      <c r="AI87" s="10" t="n"/>
+      <c r="AJ87" s="10" t="n"/>
+      <c r="AK87" s="10" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="7" t="n"/>
+      <c r="B88" s="7" t="n"/>
+      <c r="C88" s="7" t="n"/>
+      <c r="D88" s="7" t="n"/>
+      <c r="E88" s="7" t="n"/>
+      <c r="F88" s="7" t="n"/>
+      <c r="G88" s="7" t="n"/>
+      <c r="H88" s="7" t="n"/>
+      <c r="I88" s="7" t="n"/>
+      <c r="J88" s="8" t="inlineStr">
         <is>
           <t>Effective Duty Rate</t>
         </is>
       </c>
-      <c r="K87" s="7" t="n"/>
-      <c r="L87" s="7" t="n"/>
-      <c r="M87" s="7" t="n"/>
-      <c r="N87" s="7" t="n"/>
-      <c r="O87" s="7" t="n"/>
-      <c r="P87" s="12" t="n">
-        <v>0.415084885396872</v>
-      </c>
-      <c r="Q87" s="7" t="n"/>
-      <c r="R87" s="7" t="n"/>
-      <c r="S87" s="7" t="n"/>
-      <c r="T87" s="7" t="n"/>
-      <c r="U87" s="7" t="n"/>
-      <c r="V87" s="7" t="n"/>
-      <c r="W87" s="7" t="n"/>
-      <c r="X87" s="7" t="n"/>
-      <c r="Y87" s="7" t="n"/>
-      <c r="Z87" s="7" t="n"/>
-      <c r="AA87" s="7" t="n"/>
-      <c r="AB87" s="7" t="n"/>
-      <c r="AC87" s="7" t="n"/>
-      <c r="AD87" s="7" t="n"/>
-      <c r="AE87" s="7" t="n"/>
-      <c r="AF87" s="7" t="n"/>
-      <c r="AG87" s="7" t="n"/>
-      <c r="AH87" s="7" t="n"/>
-      <c r="AI87" s="7" t="n"/>
-      <c r="AJ87" s="7" t="n"/>
-      <c r="AK87" s="7" t="n"/>
+      <c r="K88" s="7" t="n"/>
+      <c r="L88" s="7" t="n"/>
+      <c r="M88" s="7" t="n"/>
+      <c r="N88" s="7" t="n"/>
+      <c r="O88" s="7" t="n"/>
+      <c r="P88" s="12" t="n">
+        <v>0.449000245996774</v>
+      </c>
+      <c r="Q88" s="7" t="n"/>
+      <c r="R88" s="7" t="n"/>
+      <c r="S88" s="7" t="n"/>
+      <c r="T88" s="7" t="n"/>
+      <c r="U88" s="7" t="n"/>
+      <c r="V88" s="7" t="n"/>
+      <c r="W88" s="7" t="n"/>
+      <c r="X88" s="7" t="n"/>
+      <c r="Y88" s="7" t="n"/>
+      <c r="Z88" s="7" t="n"/>
+      <c r="AA88" s="7" t="n"/>
+      <c r="AB88" s="7" t="n"/>
+      <c r="AC88" s="7" t="n"/>
+      <c r="AD88" s="7" t="n"/>
+      <c r="AE88" s="7" t="n"/>
+      <c r="AF88" s="7" t="n"/>
+      <c r="AG88" s="7" t="n"/>
+      <c r="AH88" s="7" t="n"/>
+      <c r="AI88" s="7" t="n"/>
+      <c r="AJ88" s="7" t="n"/>
+      <c r="AK88" s="7" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>